<commit_message>
Update training plan: Tuesday upgrade miles + corrected Floor+Upgrades weekly totals
</commit_message>
<xml_diff>
--- a/plan/uvm-training-plan.xlsx
+++ b/plan/uvm-training-plan.xlsx
@@ -1271,7 +1271,9 @@
           <t>Add 1 mi + 6 strides</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr"/>
+      <c r="H17" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -1515,7 +1517,9 @@
           <t>4 mi w/ 8x30s fartlek surges</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr"/>
+      <c r="H24" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -1759,7 +1763,9 @@
           <t>5 mi w/ 6x10s hill sprints</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr"/>
+      <c r="H31" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -2243,7 +2249,9 @@
           <t>5 mi w/ 10x(1 on / 1 off)</t>
         </is>
       </c>
-      <c r="H45" s="9" t="inlineStr"/>
+      <c r="H45" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I45" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -2731,7 +2739,9 @@
           <t>5 mi w/ 3x5 min @ tempo</t>
         </is>
       </c>
-      <c r="H59" s="9" t="inlineStr"/>
+      <c r="H59" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -2975,7 +2985,9 @@
           <t>6 mi w/ 8x45s hills</t>
         </is>
       </c>
-      <c r="H66" s="9" t="inlineStr"/>
+      <c r="H66" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I66" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -3459,7 +3471,9 @@
           <t>5 mi w/ 4x5 min @ tempo</t>
         </is>
       </c>
-      <c r="H80" s="9" t="inlineStr"/>
+      <c r="H80" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I80" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -3703,7 +3717,9 @@
           <t>6 mi w/ 20 min @ tempo</t>
         </is>
       </c>
-      <c r="H87" s="9" t="inlineStr"/>
+      <c r="H87" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I87" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -3947,7 +3963,9 @@
           <t>6 mi w/ 6x2 min @ 5K effort</t>
         </is>
       </c>
-      <c r="H94" s="9" t="inlineStr"/>
+      <c r="H94" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I94" s="9" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -4431,7 +4449,9 @@
           <t>7 mi: 6x800 @ I pace</t>
         </is>
       </c>
-      <c r="H108" s="23" t="inlineStr"/>
+      <c r="H108" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="I108" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -4675,7 +4695,9 @@
           <t>7 mi: 3x1.5 mi @ T</t>
         </is>
       </c>
-      <c r="H115" s="23" t="inlineStr"/>
+      <c r="H115" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="I115" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -4919,7 +4941,9 @@
           <t>7 mi: 5x1K @ I pace</t>
         </is>
       </c>
-      <c r="H122" s="23" t="inlineStr"/>
+      <c r="H122" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="I122" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -5163,7 +5187,9 @@
           <t>6 mi w/ 4 @ MP</t>
         </is>
       </c>
-      <c r="H129" s="23" t="inlineStr"/>
+      <c r="H129" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="I129" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -5407,7 +5433,9 @@
           <t>8 mi: 4x1 mi @ T</t>
         </is>
       </c>
-      <c r="H136" s="23" t="inlineStr"/>
+      <c r="H136" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="I136" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -5651,7 +5679,9 @@
           <t>8 mi: 6x1K @ I pace</t>
         </is>
       </c>
-      <c r="H143" s="23" t="inlineStr"/>
+      <c r="H143" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="I143" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -5895,7 +5925,9 @@
           <t>9 mi: 2x3 mi @ T</t>
         </is>
       </c>
-      <c r="H150" s="23" t="inlineStr"/>
+      <c r="H150" s="26" t="n">
+        <v>3</v>
+      </c>
       <c r="I150" s="23" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -6379,7 +6411,9 @@
           <t>9 mi: 5x1 mi @ T</t>
         </is>
       </c>
-      <c r="H164" s="33" t="inlineStr"/>
+      <c r="H164" s="36" t="n">
+        <v>3</v>
+      </c>
       <c r="I164" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -6629,7 +6663,9 @@
           <t>9 mi: 8x800 @ I pace</t>
         </is>
       </c>
-      <c r="H171" s="33" t="inlineStr"/>
+      <c r="H171" s="36" t="n">
+        <v>3</v>
+      </c>
       <c r="I171" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -6879,7 +6915,9 @@
           <t>10 mi: 3x2 mi @ T</t>
         </is>
       </c>
-      <c r="H178" s="33" t="inlineStr"/>
+      <c r="H178" s="36" t="n">
+        <v>3</v>
+      </c>
       <c r="I178" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -7129,7 +7167,9 @@
           <t>7 mi w/ 5 @ MP</t>
         </is>
       </c>
-      <c r="H185" s="33" t="inlineStr"/>
+      <c r="H185" s="36" t="n">
+        <v>2</v>
+      </c>
       <c r="I185" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -7379,7 +7419,9 @@
           <t>10 mi: 6x1K @ I + downhill finish</t>
         </is>
       </c>
-      <c r="H192" s="33" t="inlineStr"/>
+      <c r="H192" s="36" t="n">
+        <v>4</v>
+      </c>
       <c r="I192" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -7629,7 +7671,9 @@
           <t>7 mi: 3x1 mi @ half pace</t>
         </is>
       </c>
-      <c r="H199" s="33" t="inlineStr"/>
+      <c r="H199" s="36" t="n">
+        <v>2</v>
+      </c>
       <c r="I199" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -8125,7 +8169,9 @@
           <t>Upgrade LR to 22 + 10 mi: 4x1.5 @ T</t>
         </is>
       </c>
-      <c r="H213" s="33" t="inlineStr"/>
+      <c r="H213" s="36" t="n">
+        <v>3</v>
+      </c>
       <c r="I213" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -8381,7 +8427,9 @@
           <t>9 mi: 6x1K @ I pace</t>
         </is>
       </c>
-      <c r="H220" s="33" t="inlineStr"/>
+      <c r="H220" s="36" t="n">
+        <v>2</v>
+      </c>
       <c r="I220" s="33" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -8631,7 +8679,9 @@
           <t>8 mi: 5x1K @ I</t>
         </is>
       </c>
-      <c r="H227" s="43" t="inlineStr"/>
+      <c r="H227" s="46" t="n">
+        <v>2</v>
+      </c>
       <c r="I227" s="43" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -8875,7 +8925,9 @@
           <t>6 mi: 4x1 mi @ MP</t>
         </is>
       </c>
-      <c r="H234" s="43" t="inlineStr"/>
+      <c r="H234" s="46" t="n">
+        <v>1</v>
+      </c>
       <c r="I234" s="43" t="inlineStr">
         <is>
           <t>See Paces tab</t>
@@ -9455,7 +9507,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="56" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4" s="55" t="n">
         <v>5</v>
@@ -9494,7 +9546,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" s="55" t="n">
         <v>6</v>
@@ -9533,7 +9585,7 @@
         <v>16</v>
       </c>
       <c r="E6" s="56" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F6" s="55" t="n">
         <v>7</v>
@@ -9611,7 +9663,7 @@
         <v>18</v>
       </c>
       <c r="E8" s="56" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F8" s="55" t="n">
         <v>8</v>
@@ -9689,7 +9741,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F10" s="55" t="n">
         <v>9</v>
@@ -9728,7 +9780,7 @@
         <v>22</v>
       </c>
       <c r="E11" s="56" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F11" s="55" t="n">
         <v>10</v>
@@ -9806,7 +9858,7 @@
         <v>20</v>
       </c>
       <c r="E13" s="56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F13" s="55" t="n">
         <v>10</v>
@@ -9845,7 +9897,7 @@
         <v>24</v>
       </c>
       <c r="E14" s="56" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" s="55" t="n">
         <v>11</v>
@@ -9884,7 +9936,7 @@
         <v>26</v>
       </c>
       <c r="E15" s="56" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F15" s="55" t="n">
         <v>12</v>
@@ -9962,7 +10014,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="59" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F17" s="58" t="n">
         <v>13</v>
@@ -10001,7 +10053,7 @@
         <v>29</v>
       </c>
       <c r="E18" s="59" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F18" s="58" t="n">
         <v>14</v>
@@ -10040,7 +10092,7 @@
         <v>31</v>
       </c>
       <c r="E19" s="59" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" s="58" t="n">
         <v>15</v>
@@ -10079,7 +10131,7 @@
         <v>25</v>
       </c>
       <c r="E20" s="59" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F20" s="58" t="n">
         <v>12</v>
@@ -10118,7 +10170,7 @@
         <v>32</v>
       </c>
       <c r="E21" s="59" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F21" s="58" t="n">
         <v>16</v>
@@ -10157,7 +10209,7 @@
         <v>34</v>
       </c>
       <c r="E22" s="59" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F22" s="58" t="n">
         <v>17</v>
@@ -10196,7 +10248,7 @@
         <v>35</v>
       </c>
       <c r="E23" s="59" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F23" s="58" t="n">
         <v>18</v>
@@ -10274,7 +10326,7 @@
         <v>36</v>
       </c>
       <c r="E25" s="61" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F25" s="60" t="n">
         <v>18</v>
@@ -10313,7 +10365,7 @@
         <v>38</v>
       </c>
       <c r="E26" s="61" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F26" s="60" t="n">
         <v>20</v>
@@ -10352,7 +10404,7 @@
         <v>39</v>
       </c>
       <c r="E27" s="61" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F27" s="60" t="n">
         <v>16</v>
@@ -10391,7 +10443,7 @@
         <v>30</v>
       </c>
       <c r="E28" s="61" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F28" s="60" t="n">
         <v>13</v>
@@ -10430,7 +10482,7 @@
         <v>38</v>
       </c>
       <c r="E29" s="61" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F29" s="60" t="n">
         <v>18</v>
@@ -10469,7 +10521,7 @@
         <v>30</v>
       </c>
       <c r="E30" s="57" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F30" s="57" t="n">
         <v>13.1</v>
@@ -10547,7 +10599,7 @@
         <v>40</v>
       </c>
       <c r="E32" s="61" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F32" s="60" t="n">
         <v>20</v>
@@ -10586,7 +10638,7 @@
         <v>38</v>
       </c>
       <c r="E33" s="61" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F33" s="60" t="n">
         <v>16</v>
@@ -10625,7 +10677,7 @@
         <v>32</v>
       </c>
       <c r="E34" s="63" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F34" s="62" t="n">
         <v>13</v>
@@ -10664,7 +10716,7 @@
         <v>24</v>
       </c>
       <c r="E35" s="63" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F35" s="62" t="n">
         <v>10</v>

</xml_diff>